<commit_message>
auto: snapshot 2026-07-16 13:01:01
</commit_message>
<xml_diff>
--- a/crew_101.xlsx
+++ b/crew_101.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-15" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1417,4 +1418,990 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew: Shad0w Ninjas (101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-16 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Dmg</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Dmg</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Boss Kills</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Kills</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>448708</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+165576</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2134</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>356048</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+98759</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1697</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>331994</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+83880</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1582</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>516348</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+153261</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>2458</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>437820</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+166336</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>2086</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>424481</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+153298</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>228266</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+24564</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>1088</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>367206</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+142165</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>1748</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>375185</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+181876</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1786</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>340858</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+87061</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1624</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>567835</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+198660</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>2703</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>389013</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+82830</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1852</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>349977</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+88442</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>1596</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>485363</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+67468</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>2310</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>340778</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+85710</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>1551</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>272747</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+64666</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>321443</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+85827</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>1458</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>657944</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+149384</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>3133</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>630629</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+241474</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>3002</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>337564</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+88250</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1534</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>612668</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+182961</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>2918</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>373245</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+79230</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>1776</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>236736</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+78916</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>1128</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>416120</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+85068</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>590191</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+144049</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>2809</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>297978</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+78688</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>1418</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>408518</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+131703</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>1945</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Lovebird | Gorelax</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>329669</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+88726</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>1495</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>547330</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+200745</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>2605</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>569916</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+258955</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>2716</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>459836</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+145612</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>2190</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>360091</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+98678</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>1716</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>544177</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+132271</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>2586</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>403896</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+81739</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>1923</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>710626</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+320779</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>3373</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>659024</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+237122</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>3138</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>423335</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+145291</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>390932</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+74219</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>1862</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>318674</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+85502</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>1445</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>474739</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>2255</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-18 13:01:01
</commit_message>
<xml_diff>
--- a/crew_101.xlsx
+++ b/crew_101.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-07-15" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-17" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-18" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3391,4 +3392,990 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew: Shad0w Ninjas (101) | S28 P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-18 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Dmg</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Dmg</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Boss Kills</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Kills</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>680359</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+115945</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>3238</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>+1094</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>586316</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+115733</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>2794</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>+1087</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>505190</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+95875</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>2407</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>+752</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>713541</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+116030</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>3396</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>+928</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>652017</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+113100</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>3107</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>+1011</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>677046</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+117657</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>3224</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>+1193</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>517876</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+151296</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>2466</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>+1377</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>614959</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+118983</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>2930</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>+1172</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>506241</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+80795</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>2410</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>+621</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>535394</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+96237</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>2552</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>+852</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>737511</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+89114</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>3511</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+798</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>627036</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+116334</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>2987</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>557217</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+109782</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>2583</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>+977</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>664827</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+87676</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>3164</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+844</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>531348</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+93214</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>2459</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+898</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>475617</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+69488</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>2266</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>+966</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>527358</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+109735</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>2438</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>+970</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>977946</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+107913</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>4656</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+1480</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>790123</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+96266</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>3762</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+758</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>540445</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+108654</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>2501</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>+957</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>871787</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+93474</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>4153</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>+1185</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>606316</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+116220</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>2886</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>510389</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+142869</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>2430</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>+1302</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>648816</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+116001</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>3092</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>+1098</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1284632</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+190175</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>6118</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>+3273</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>457246</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+97812</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>2177</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>+749</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>640814</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+115910</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>3051</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>+1096</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Lovebird | Gorelax</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>536249</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+109627</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>2480</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>812904</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+87597</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>3870</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>+1218</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>816842</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+88099</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>3890</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>+1137</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>682486</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+98603</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>3249</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>+1049</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>613941</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+115924</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>2924</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>+1198</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>754633</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+145914</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>3588</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>+992</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>637942</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+172034</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>3036</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>+1113</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>990625</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+115660</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>4704</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>+1283</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>896666</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+111348</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>4268</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>+1106</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>674442</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+114317</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>3211</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>+1185</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>637433</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+143424</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>3036</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>+1163</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>521534</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+107206</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>2412</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>+957</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>660684</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>3141</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>+886</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>